<commit_message>
before: fix protein card white background for eggs and prawns
</commit_message>
<xml_diff>
--- a/Recipes/input/recipe_template_onboarded.xlsx
+++ b/Recipes/input/recipe_template_onboarded.xlsx
@@ -8,22 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\v_gow\SpiceStrong\Recipes\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C0BDA75E-59FA-484F-BBB7-0171E007C587}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F1B9E74-DA96-49C4-B3F2-335C2B433B1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2715" yWindow="2910" windowWidth="18810" windowHeight="17145" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4290" yWindow="4290" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Recipe Info" sheetId="1" r:id="rId1"/>
     <sheet name="Ingredients" sheetId="2" r:id="rId2"/>
     <sheet name="Cooking Steps" sheetId="3" r:id="rId3"/>
-    <sheet name="Nutrition" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
   <si>
     <t>Field</t>
   </si>
@@ -67,9 +66,6 @@
     <t>Gluten Free</t>
   </si>
   <si>
-    <t>Fitness Friendly</t>
-  </si>
-  <si>
     <t>Cooking Method</t>
   </si>
   <si>
@@ -101,15 +97,6 @@
   </si>
   <si>
     <t>Chef Tip</t>
-  </si>
-  <si>
-    <t>Nutrient</t>
-  </si>
-  <si>
-    <t>Per Serving (2–3 Servings)</t>
-  </si>
-  <si>
-    <t>Per Serving (4–6 Servings)</t>
   </si>
 </sst>
 </file>
@@ -455,7 +442,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="38" customWidth="1"/>
@@ -534,11 +521,6 @@
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>15</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -546,7 +528,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="28" customWidth="1"/>
@@ -554,16 +536,106 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>19</v>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -581,49 +653,25 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="3" width="30" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>